<commit_message>
B&N rev9 WIP: C8-01..C8-08 applied (slab pins, #8 screws 8/A-410, track split by size, purchase units, S-12 base), skill v80p R80e.31
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UQBQT8jCVU6KW8QmKhZS83
</commit_message>
<xml_diff>
--- a/cache_proyectos/barnes_noble/PASO12_rev7/MATRIZ_COBERTURA.xlsx
+++ b/cache_proyectos/barnes_noble/PASO12_rev7/MATRIZ_COBERTURA.xlsx
@@ -25196,7 +25196,7 @@
       </c>
       <c r="H485" s="2" t="inlineStr">
         <is>
-          <t>C7-03: + P.A.F. 3/16" x 3/8" 282 pcs [DERIVED 705.0 / 5.0 = 141 members x 2]; #8 screws covered by framing screws.</t>
+          <t>C7-03: + P.A.F. 3/16" x 3/8" 282 pcs [DERIVED 705.0 / 5.0 = 141 members x 2]; #8 screws covered by framing screws. [CORRECTED rev9: false - framing screws count stud pieces only; the 8/A-410 #8 screws now have their own row, 775 pcs]</t>
         </is>
       </c>
       <c r="I485" s="2" t="inlineStr"/>
@@ -27497,7 +27497,7 @@
         <v>278.57</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>6964.25</v>

</xml_diff>